<commit_message>
update wo and fix bug
</commit_message>
<xml_diff>
--- a/Template_Outage_EIC_Monitoring_unit 1.xlsx
+++ b/Template_Outage_EIC_Monitoring_unit 1.xlsx
@@ -1029,14 +1029,9 @@
           <t>22/08/2026</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>29/08/2026</t>
-        </is>
-      </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>FINISH</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -1048,7 +1043,7 @@
         <v>9</v>
       </c>
       <c r="L2" t="n">
-        <v>100</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -1390,7 +1385,7 @@
         <v>17</v>
       </c>
       <c r="L8" t="n">
-        <v>76.5</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1442,7 +1437,7 @@
         <v>12</v>
       </c>
       <c r="L9" t="n">
-        <v>16.7</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1499,7 +1494,7 @@
         <v>12</v>
       </c>
       <c r="L10" t="n">
-        <v>75</v>
+        <v>91.7</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1556,7 +1551,7 @@
         <v>6</v>
       </c>
       <c r="L11" t="n">
-        <v>66.7</v>
+        <v>33.3</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1670,7 +1665,7 @@
         <v>6</v>
       </c>
       <c r="L13" t="n">
-        <v>83.3</v>
+        <v>33.3</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1727,7 +1722,7 @@
         <v>11</v>
       </c>
       <c r="L14" t="n">
-        <v>72.7</v>
+        <v>81.8</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1767,7 +1762,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1779,7 +1774,7 @@
         <v>7</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>28.6</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -2097,7 +2092,6 @@
           <t>22/08/2026</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>IN PROGRESS</t>
@@ -2119,7 +2113,6 @@
           <t>SUPERVISE, QC, OTHER TASK AS PER EIC JP</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
       <c r="Q21" t="n">
         <v>0</v>
       </c>
@@ -2351,7 +2344,7 @@
         <v>32</v>
       </c>
       <c r="L25" t="n">
-        <v>28.1</v>
+        <v>34.4</v>
       </c>
       <c r="M25" t="inlineStr">
         <is>
@@ -2465,7 +2458,7 @@
         <v>12</v>
       </c>
       <c r="L27" t="n">
-        <v>33.3</v>
+        <v>58.3</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
@@ -2522,7 +2515,7 @@
         <v>7</v>
       </c>
       <c r="L28" t="n">
-        <v>57.1</v>
+        <v>85.7</v>
       </c>
       <c r="M28" t="inlineStr">
         <is>
@@ -2579,7 +2572,7 @@
         <v>7</v>
       </c>
       <c r="L29" t="n">
-        <v>57.1</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="M29" t="inlineStr">
         <is>
@@ -2728,7 +2721,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2740,7 +2733,7 @@
         <v>24</v>
       </c>
       <c r="L32" t="n">
-        <v>0</v>
+        <v>12.5</v>
       </c>
       <c r="M32" t="inlineStr">
         <is>
@@ -2901,7 +2894,7 @@
         <v>56</v>
       </c>
       <c r="L35" t="n">
-        <v>10.7</v>
+        <v>17.9</v>
       </c>
       <c r="M35" t="inlineStr">
         <is>
@@ -2996,6 +2989,11 @@
           <t>22/08/2026</t>
         </is>
       </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>FINISH</t>
@@ -3162,9 +3160,14 @@
           <t>22/08/2026</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -3176,7 +3179,7 @@
         <v>18</v>
       </c>
       <c r="L40" t="n">
-        <v>33.3</v>
+        <v>100</v>
       </c>
       <c r="M40" t="inlineStr">
         <is>
@@ -3233,7 +3236,7 @@
         <v>21</v>
       </c>
       <c r="L41" t="n">
-        <v>57.1</v>
+        <v>66.7</v>
       </c>
       <c r="M41" t="inlineStr">
         <is>
@@ -4356,9 +4359,14 @@
           <t>22/08/2026</t>
         </is>
       </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -4370,7 +4378,7 @@
         <v>12</v>
       </c>
       <c r="L62" t="n">
-        <v>91.7</v>
+        <v>100</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
@@ -4422,7 +4430,7 @@
         <v>5</v>
       </c>
       <c r="L63" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="M63" t="inlineStr">
         <is>
@@ -4465,9 +4473,14 @@
           <t>22/08/2026</t>
         </is>
       </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -4479,13 +4492,14 @@
         <v>6</v>
       </c>
       <c r="L64" t="n">
-        <v>83.3</v>
+        <v>100</v>
       </c>
       <c r="M64" t="inlineStr">
         <is>
           <t>SUPERVISE, QC, OTHER TASK AS PER EIC JP</t>
         </is>
       </c>
+      <c r="N64" t="inlineStr"/>
       <c r="Q64" t="n">
         <v>0</v>
       </c>
@@ -4848,18 +4862,13 @@
           <t>SOLO RUN</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>29/08/2026</t>
-        </is>
-      </c>
       <c r="D10" t="inlineStr">
         <is>
           <t>H AIDI</t>
         </is>
       </c>
       <c r="E10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
         <v>0</v>
@@ -6032,7 +6041,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>30/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -6060,7 +6069,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>30/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -6312,7 +6321,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -6417,18 +6426,13 @@
           <t>UNIT 1 INDUCED DRAUGHT FAN 2 INLET ACTUATOR MOV 20HNA62AA001</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>30/08/2026</t>
-        </is>
-      </c>
       <c r="D68" t="inlineStr">
         <is>
           <t>AMP</t>
         </is>
       </c>
       <c r="E68" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H68" t="n">
         <v>0</v>
@@ -7034,18 +7038,13 @@
           <t>20HLB01CP104: LO HEADER PRESSURE LOW ALARM FOR PA FAN-1</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
       <c r="D92" t="inlineStr">
         <is>
           <t>H AIDI</t>
         </is>
       </c>
       <c r="E92" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H92" t="n">
         <v>0</v>
@@ -7062,18 +7061,13 @@
           <t>20HLB01CP103: PRESSURE SWITCH TO START PERMISSIVE FOR PA FAN-1 START</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
       <c r="D93" t="inlineStr">
         <is>
           <t>H AIDI</t>
         </is>
       </c>
       <c r="E93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H93" t="n">
         <v>0</v>
@@ -7467,18 +7461,13 @@
           <t>20HLB02CP104: LO HEADER PRESSURE LOW ALARM FOR PA FAN-2</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
       <c r="D108" t="inlineStr">
         <is>
           <t>H AIDI</t>
         </is>
       </c>
       <c r="E108" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H108" t="n">
         <v>0</v>
@@ -7495,18 +7484,13 @@
           <t>20HLB02CP103: PRESSURE SWITCH TO START PERMISSIVE FOR PA FAN-2 START</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
       <c r="D109" t="inlineStr">
         <is>
           <t>H AIDI</t>
         </is>
       </c>
       <c r="E109" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H109" t="n">
         <v>0</v>
@@ -7523,18 +7507,13 @@
           <t>20HLB02CP102: PRESSURE SWITCH TO START LO PA FAN-2 STANDBY PUMP</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
       <c r="D110" t="inlineStr">
         <is>
           <t>H AIDI</t>
         </is>
       </c>
       <c r="E110" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H110" t="n">
         <v>0</v>
@@ -7844,13 +7823,18 @@
           <t>MSW20HLN10-M101:UNIT 1 SECONDARY AIR FAN 1 LUBE OIL PUMP 1 MOTOR (STAND BY)</t>
         </is>
       </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D122" t="inlineStr">
         <is>
           <t>H AIDI</t>
         </is>
       </c>
       <c r="E122" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H122" t="n">
         <v>0</v>
@@ -7867,13 +7851,18 @@
           <t>MSW20HLN10-M102:UNIT 1 SECONDARY AIR FAN 1 LUBE OIL PUMP 2 MOTOR (MAIN)</t>
         </is>
       </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D123" t="inlineStr">
         <is>
           <t>H AIDI</t>
         </is>
       </c>
       <c r="E123" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H123" t="n">
         <v>0</v>
@@ -11853,18 +11842,13 @@
           <t>UNIT 1 FEED WATER INLET ECONOMIZER MOTORIZED VALVE ISOLATION VALVE</t>
         </is>
       </c>
-      <c r="C280" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
       <c r="D280" t="inlineStr">
         <is>
           <t>AMP</t>
         </is>
       </c>
       <c r="E280" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H280" t="n">
         <v>0</v>
@@ -11973,13 +11957,18 @@
           <t>DISTRIBUTOR LINE TO FEEDWATER TRANSMITTER 10LAB30CP001</t>
         </is>
       </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D285" t="inlineStr">
         <is>
           <t>JAPA</t>
         </is>
       </c>
       <c r="E285" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H285" t="n">
         <v>0</v>
@@ -11996,13 +11985,18 @@
           <t>INLET FEEDWATER PRESSURE TRANSMITTER 10HAC90CP001</t>
         </is>
       </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D286" t="inlineStr">
         <is>
           <t>JAPA</t>
         </is>
       </c>
       <c r="E286" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H286" t="n">
         <v>0</v>
@@ -12019,13 +12013,18 @@
           <t>INLET FEEDWATER FLOW TRANSMITTER 10HAC90CF001</t>
         </is>
       </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D287" t="inlineStr">
         <is>
           <t>JAPA</t>
         </is>
       </c>
       <c r="E287" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H287" t="n">
         <v>0</v>
@@ -12042,13 +12041,18 @@
           <t>INLET FEEDWATER FLOW TRANSMITTER 10HAC90CF002</t>
         </is>
       </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D288" t="inlineStr">
         <is>
           <t>JAPA</t>
         </is>
       </c>
       <c r="E288" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H288" t="n">
         <v>0</v>
@@ -14290,13 +14294,18 @@
           <t>INSPECTION BOLT BUSBAR, FLANGE &amp; INSPECTION HOLE BUSDUCT</t>
         </is>
       </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D384" t="inlineStr">
         <is>
           <t>JAPA</t>
         </is>
       </c>
       <c r="E384" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H384" t="n">
         <v>0</v>
@@ -14336,13 +14345,18 @@
           <t>CEK KEBOCORAN DAN KELEMBAPAN BUSDUCT</t>
         </is>
       </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D386" t="inlineStr">
         <is>
           <t>JAPA</t>
         </is>
       </c>
       <c r="E386" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H386" t="n">
         <v>0</v>
@@ -14405,13 +14419,18 @@
           <t>CLEANING</t>
         </is>
       </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D389" t="inlineStr">
         <is>
           <t>JAPA</t>
         </is>
       </c>
       <c r="E389" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H389" t="n">
         <v>0</v>
@@ -15008,13 +15027,18 @@
           <t>CONDENSATE PRESSURE TO BYPASS SPRAY PRESSURE TRANSMITTER (20LCE40CP001)</t>
         </is>
       </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D415" t="inlineStr">
         <is>
           <t>M TOHER</t>
         </is>
       </c>
       <c r="E415" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H415" t="n">
         <v>0</v>
@@ -15031,13 +15055,18 @@
           <t>CONDENSATE PRESSURE TO BYPASS SPRAY PRESSURE TRANSMITTER (20LCE40CP002)</t>
         </is>
       </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D416" t="inlineStr">
         <is>
           <t>M TOHER</t>
         </is>
       </c>
       <c r="E416" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H416" t="n">
         <v>0</v>
@@ -15054,13 +15083,18 @@
           <t>CONDENSATE PRESSURE TO BYPASS SPRAY PRESSURE TRANSMITTER (20LCE40CP003)</t>
         </is>
       </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D417" t="inlineStr">
         <is>
           <t>M TOHER</t>
         </is>
       </c>
       <c r="E417" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H417" t="n">
         <v>0</v>
@@ -16310,7 +16344,7 @@
       </c>
       <c r="C470" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>29/08/2026</t>
         </is>
       </c>
       <c r="D470" t="inlineStr">
@@ -16338,7 +16372,7 @@
       </c>
       <c r="C471" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>29/08/2026</t>
         </is>
       </c>
       <c r="D471" t="inlineStr">
@@ -16394,7 +16428,7 @@
       </c>
       <c r="C473" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D473" t="inlineStr">
@@ -16672,7 +16706,7 @@
       </c>
       <c r="C484" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D484" t="inlineStr">
@@ -16700,7 +16734,7 @@
       </c>
       <c r="C485" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D485" t="inlineStr">
@@ -16728,7 +16762,7 @@
       </c>
       <c r="C486" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D486" t="inlineStr">
@@ -16838,13 +16872,18 @@
           <t>DRUM LEVEL TRANSMITTER 10HAD10CL001</t>
         </is>
       </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D490" t="inlineStr">
         <is>
           <t>JHON</t>
         </is>
       </c>
       <c r="E490" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H490" t="n">
         <v>0</v>
@@ -16861,13 +16900,18 @@
           <t>DRUM LEVEL TRANSMITTER 10HAD10CL002</t>
         </is>
       </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D491" t="inlineStr">
         <is>
           <t>JHON</t>
         </is>
       </c>
       <c r="E491" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H491" t="n">
         <v>0</v>
@@ -16884,13 +16928,18 @@
           <t>DRUM LEVEL TRANSMITTER 10HAD10CL003</t>
         </is>
       </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D492" t="inlineStr">
         <is>
           <t>JHON</t>
         </is>
       </c>
       <c r="E492" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H492" t="n">
         <v>0</v>
@@ -16907,13 +16956,18 @@
           <t>DRUM PRESSURE TRANSMITTER 10HAD10CP002</t>
         </is>
       </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D493" t="inlineStr">
         <is>
           <t>JHON</t>
         </is>
       </c>
       <c r="E493" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H493" t="n">
         <v>0</v>
@@ -16930,13 +16984,18 @@
           <t>DRUM PRESSURE TRANSMITTER 10HAD10CP003</t>
         </is>
       </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D494" t="inlineStr">
         <is>
           <t>JHON</t>
         </is>
       </c>
       <c r="E494" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H494" t="n">
         <v>0</v>
@@ -16953,13 +17012,18 @@
           <t>DRUM PRESSURE TRANSMITTER 10HAD10CP001</t>
         </is>
       </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D495" t="inlineStr">
         <is>
           <t>JHON</t>
         </is>
       </c>
       <c r="E495" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H495" t="n">
         <v>0</v>
@@ -17345,7 +17409,7 @@
       </c>
       <c r="C510" t="inlineStr">
         <is>
-          <t>29/8/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="D510" t="inlineStr">
@@ -17373,7 +17437,7 @@
       </c>
       <c r="C511" t="inlineStr">
         <is>
-          <t>29/8/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="D511" t="inlineStr">
@@ -17401,7 +17465,7 @@
       </c>
       <c r="C512" t="inlineStr">
         <is>
-          <t>29/8/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="D512" t="inlineStr">
@@ -17427,13 +17491,18 @@
           <t>BACKPASS PRESSURE AFTER LT SH TRANSMITTER 10HBK01CP030</t>
         </is>
       </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
+        </is>
+      </c>
       <c r="D513" t="inlineStr">
         <is>
           <t>M TOHER</t>
         </is>
       </c>
       <c r="E513" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H513" t="n">
         <v>0</v>
@@ -17450,13 +17519,18 @@
           <t>BACKPASS PRESSURE AFTER ECO TRANSMITTER 10HBK01CP050</t>
         </is>
       </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D514" t="inlineStr">
         <is>
           <t>M TOHER</t>
         </is>
       </c>
       <c r="E514" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H514" t="n">
         <v>0</v>
@@ -22104,13 +22178,18 @@
           <t>HOUSEKEEPING</t>
         </is>
       </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="D702" t="inlineStr">
         <is>
           <t>JAPA</t>
         </is>
       </c>
       <c r="E702" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H702" t="n">
         <v>0</v>
@@ -22173,18 +22252,13 @@
           <t>ACTUATOR GLAND STEAM PRESSURE CONTROL VALVE 10MAW10AA210</t>
         </is>
       </c>
-      <c r="C705" t="inlineStr">
-        <is>
-          <t>29/8/2026</t>
-        </is>
-      </c>
       <c r="D705" t="inlineStr">
         <is>
           <t>H AIDI</t>
         </is>
       </c>
       <c r="E705" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H705" t="n">
         <v>0</v>
@@ -22389,21 +22463,26 @@
     <row r="713">
       <c r="A713" t="inlineStr">
         <is>
-          <t>WO-100826-0074</t>
+          <t>WO-100826-0075</t>
         </is>
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>BACKPASS PRESSURE AFTER ECO TRANSMITTER</t>
+          <t>Panel Bapcon - Rapcon Field 1</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="D713" t="inlineStr">
         <is>
-          <t>FERRYUS</t>
+          <t>M IQBAL</t>
         </is>
       </c>
       <c r="E713" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H713" t="n">
         <v>0</v>
@@ -22417,7 +22496,7 @@
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>Panel Bapcon - Rapcon Field 1</t>
+          <t>Panel Bapcon - Rapcon Field 2</t>
         </is>
       </c>
       <c r="C714" t="inlineStr">
@@ -22445,12 +22524,12 @@
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>Panel Bapcon - Rapcon Field 2</t>
+          <t>Panel Bapcon - Rapcon Field 3</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>29/8/2026</t>
         </is>
       </c>
       <c r="D715" t="inlineStr">
@@ -22473,12 +22552,7 @@
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>Panel Bapcon - Rapcon Field 3</t>
-        </is>
-      </c>
-      <c r="C716" t="inlineStr">
-        <is>
-          <t>29/8/2026</t>
+          <t>Panel Bapcon - Rapcon Field 4</t>
         </is>
       </c>
       <c r="D716" t="inlineStr">
@@ -22487,7 +22561,7 @@
         </is>
       </c>
       <c r="E716" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H716" t="n">
         <v>0</v>
@@ -22501,7 +22575,7 @@
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>Panel Bapcon - Rapcon Field 4</t>
+          <t>Panel Bapcon - Rapcon Field 5</t>
         </is>
       </c>
       <c r="D717" t="inlineStr">
@@ -22524,7 +22598,7 @@
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>Panel Bapcon - Rapcon Field 5</t>
+          <t>Panel Bapcon - Rapcon Field 6</t>
         </is>
       </c>
       <c r="D718" t="inlineStr">
@@ -22542,21 +22616,21 @@
     <row r="719">
       <c r="A719" t="inlineStr">
         <is>
-          <t>WO-100826-0075</t>
+          <t>WO-100826-0059</t>
         </is>
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>Panel Bapcon - Rapcon Field 6</t>
-        </is>
-      </c>
-      <c r="D719" t="inlineStr">
-        <is>
-          <t>M IQBAL</t>
+          <t>MOV MAIN STEAM DRAIN</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="E719" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H719" t="n">
         <v>0</v>
@@ -22565,17 +22639,22 @@
     <row r="720">
       <c r="A720" t="inlineStr">
         <is>
-          <t>WO-100826-0059</t>
+          <t>WO-100826-0038</t>
         </is>
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>MOV MAIN STEAM DRAIN</t>
+          <t>ACTUATOR DESH-1 SPRAY WATER ISOLATION</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
         <is>
-          <t>29/8/2026</t>
+          <t>29/08/2026</t>
+        </is>
+      </c>
+      <c r="D720" t="inlineStr">
+        <is>
+          <t>AMP</t>
         </is>
       </c>
       <c r="E720" t="b">
@@ -22588,17 +22667,12 @@
     <row r="721">
       <c r="A721" t="inlineStr">
         <is>
-          <t>WO-100826-0038</t>
+          <t>WO-100826-0039</t>
         </is>
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>ACTUATOR DESH-1 SPRAY WATER ISOLATION</t>
-        </is>
-      </c>
-      <c r="C721" t="inlineStr">
-        <is>
-          <t>29/08/2026</t>
+          <t>ACTUATOR DESH-2 SPRAY WATER ISOLATION</t>
         </is>
       </c>
       <c r="D721" t="inlineStr">
@@ -22607,7 +22681,7 @@
         </is>
       </c>
       <c r="E721" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H721" t="n">
         <v>0</v>
@@ -22616,12 +22690,17 @@
     <row r="722">
       <c r="A722" t="inlineStr">
         <is>
-          <t>WO-100826-0039</t>
+          <t>WO-100826-0160</t>
         </is>
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>ACTUATOR DESH-2 SPRAY WATER ISOLATION</t>
+          <t>ACTUATOR INLET ID FAN 1 MOV 10HNA61AA001</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D722" t="inlineStr">
@@ -22630,7 +22709,7 @@
         </is>
       </c>
       <c r="E722" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H722" t="n">
         <v>0</v>
@@ -22644,7 +22723,7 @@
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>ACTUATOR INLET ID FAN 1 MOV 10HNA61AA001</t>
+          <t>ACTUATOR OUTLET ID FAN 1 MOV 10HNA71AA001</t>
         </is>
       </c>
       <c r="D723" t="inlineStr">
@@ -22662,21 +22741,26 @@
     <row r="724">
       <c r="A724" t="inlineStr">
         <is>
-          <t>WO-100826-0160</t>
+          <t>WO-100826-0020</t>
         </is>
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>ACTUATOR OUTLET ID FAN 1 MOV 10HNA71AA001</t>
+          <t>ACTUATOR MOV OUTLET PA FAN 1</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D724" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>MSW</t>
         </is>
       </c>
       <c r="E724" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H724" t="n">
         <v>0</v>
@@ -22690,7 +22774,12 @@
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>ACTUATOR MOV OUTLET PA FAN 1</t>
+          <t>ACTUATOR MOV PA FAN 1</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D725" t="inlineStr">
@@ -22699,7 +22788,7 @@
         </is>
       </c>
       <c r="E725" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H725" t="n">
         <v>0</v>
@@ -22708,12 +22797,17 @@
     <row r="726">
       <c r="A726" t="inlineStr">
         <is>
-          <t>WO-100826-0020</t>
+          <t>WO-100826-0035</t>
         </is>
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>ACTUATOR MOV PA FAN 1</t>
+          <t>ACTUATOR ISOLATION STARTUP VENTING BOILER</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D726" t="inlineStr">
@@ -22722,7 +22816,7 @@
         </is>
       </c>
       <c r="E726" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H726" t="n">
         <v>0</v>
@@ -22731,12 +22825,17 @@
     <row r="727">
       <c r="A727" t="inlineStr">
         <is>
-          <t>WO-100826-0035</t>
+          <t>WO-100826-0026</t>
         </is>
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>ACTUATOR ISOLATION STARTUP VENTING BOILER</t>
+          <t>ACTUATOR IGV SA FAN 2 10HLB02EX001</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
         </is>
       </c>
       <c r="D727" t="inlineStr">
@@ -22745,7 +22844,7 @@
         </is>
       </c>
       <c r="E727" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H727" t="n">
         <v>0</v>
@@ -22754,17 +22853,12 @@
     <row r="728">
       <c r="A728" t="inlineStr">
         <is>
-          <t>WO-100826-0026</t>
+          <t>WO-100826-0035</t>
         </is>
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>ACTUATOR IGV SA FAN 2 10HLB02EX001</t>
-        </is>
-      </c>
-      <c r="C728" t="inlineStr">
-        <is>
-          <t>30/08/2026</t>
+          <t>ACTUATOR IGV SA CONTROL DAMPER 10HLA25AA010</t>
         </is>
       </c>
       <c r="D728" t="inlineStr">
@@ -22773,7 +22867,7 @@
         </is>
       </c>
       <c r="E728" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H728" t="n">
         <v>0</v>
@@ -22787,7 +22881,7 @@
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>ACTUATOR IGV SA CONTROL DAMPER 10HLA25AA010</t>
+          <t>ACTUATOR IGV SUB 1 10HJL10AA010</t>
         </is>
       </c>
       <c r="D729" t="inlineStr">
@@ -22810,7 +22904,7 @@
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>ACTUATOR IGV SUB 1 10HJL10AA010</t>
+          <t>ACTUATOR IGV SUB 2 10HJL11AA010</t>
         </is>
       </c>
       <c r="D730" t="inlineStr">
@@ -22828,12 +22922,12 @@
     <row r="731">
       <c r="A731" t="inlineStr">
         <is>
-          <t>WO-100826-0035</t>
+          <t>WO-100826-0051</t>
         </is>
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>ACTUATOR IGV SUB 2 10HJL11AA010</t>
+          <t>FLUIDIZING VALVE BED MATERIAL</t>
         </is>
       </c>
       <c r="D731" t="inlineStr">
@@ -22856,7 +22950,7 @@
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>FLUIDIZING VALVE BED MATERIAL</t>
+          <t>FLUIDIZING VALVE LIMESTONE 1&amp;2</t>
         </is>
       </c>
       <c r="D732" t="inlineStr">
@@ -22874,12 +22968,17 @@
     <row r="733">
       <c r="A733" t="inlineStr">
         <is>
-          <t>WO-100826-0051</t>
+          <t>WO-100826-0050</t>
         </is>
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>FLUIDIZING VALVE LIMESTONE 1&amp;2</t>
+          <t>ACTUATOR STEAM DRUM VENTING ISOLATION VALVE</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D733" t="inlineStr">
@@ -22888,7 +22987,7 @@
         </is>
       </c>
       <c r="E733" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H733" t="n">
         <v>0</v>
@@ -22902,7 +23001,12 @@
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>ACTUATOR STEAM DRUM VENTING ISOLATION VALVE</t>
+          <t>ACTUATOR STEAM DRUM MOV VENTING VALVE</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D734" t="inlineStr">
@@ -22911,7 +23015,7 @@
         </is>
       </c>
       <c r="E734" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H734" t="n">
         <v>0</v>
@@ -22925,7 +23029,12 @@
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>ACTUATOR STEAM DRUM MOV VENTING VALVE</t>
+          <t>ACTUATOR STEAM DRUM CBD ISOLATION VALVE</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D735" t="inlineStr">
@@ -22934,7 +23043,7 @@
         </is>
       </c>
       <c r="E735" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H735" t="n">
         <v>0</v>
@@ -22948,7 +23057,12 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>ACTUATOR STEAM DRUM CBD ISOLATION VALVE</t>
+          <t>ACTUATOR STEAM DRUM MOV CBD CONTROL VALVE</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D736" t="inlineStr">
@@ -22957,7 +23071,7 @@
         </is>
       </c>
       <c r="E736" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H736" t="n">
         <v>0</v>
@@ -22971,7 +23085,12 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>ACTUATOR STEAM DRUM MOV CBD CONTROL VALVE</t>
+          <t>ACTUATOR STEAM DRUM IBD ISOLATION VALVE</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D737" t="inlineStr">
@@ -22980,7 +23099,7 @@
         </is>
       </c>
       <c r="E737" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H737" t="n">
         <v>0</v>
@@ -22994,7 +23113,12 @@
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>ACTUATOR STEAM DRUM IBD ISOLATION VALVE</t>
+          <t>ACTUATOR STEAM DRUM MOV IBD CONTROL VALVE</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D738" t="inlineStr">
@@ -23003,7 +23127,7 @@
         </is>
       </c>
       <c r="E738" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H738" t="n">
         <v>0</v>
@@ -23012,12 +23136,17 @@
     <row r="739">
       <c r="A739" t="inlineStr">
         <is>
-          <t>WO-100826-0050</t>
+          <t>WO-100826-0035</t>
         </is>
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>ACTUATOR STEAM DRUM MOV IBD CONTROL VALVE</t>
+          <t>ACTUATOR MOV PA FAN2</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D739" t="inlineStr">
@@ -23026,7 +23155,7 @@
         </is>
       </c>
       <c r="E739" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H739" t="n">
         <v>0</v>
@@ -23035,12 +23164,17 @@
     <row r="740">
       <c r="A740" t="inlineStr">
         <is>
-          <t>WO-100826-0035</t>
+          <t>WO-100826-0024</t>
         </is>
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>ACTUATOR MOV PA FAN2</t>
+          <t>ACTUATOR MOV OUTLET SA FAN 1</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D740" t="inlineStr">
@@ -23049,7 +23183,7 @@
         </is>
       </c>
       <c r="E740" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H740" t="n">
         <v>0</v>
@@ -23058,12 +23192,12 @@
     <row r="741">
       <c r="A741" t="inlineStr">
         <is>
-          <t>WO-100826-0024</t>
+          <t>WO-100826-0058</t>
         </is>
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>ACTUATOR MOV OUTLET SA FAN 1</t>
+          <t>ACTUATOR HP BYPASS CONTROL VALVE 10LBF10AA210</t>
         </is>
       </c>
       <c r="D741" t="inlineStr">
@@ -23086,7 +23220,7 @@
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>ACTUATOR HP BYPASS CONTROL VALVE 10LBF10AA210</t>
+          <t>ACTUATOR BYPASS SPRAY CONTROL VALVE 10LCE40AA210</t>
         </is>
       </c>
       <c r="D742" t="inlineStr">
@@ -23104,12 +23238,12 @@
     <row r="743">
       <c r="A743" t="inlineStr">
         <is>
-          <t>WO-100826-0058</t>
+          <t>WO-100826-0045</t>
         </is>
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>ACTUATOR BYPASS SPRAY CONTROL VALVE 10LCE40AA210</t>
+          <t>CEP DISCHARGE VALVE</t>
         </is>
       </c>
       <c r="D743" t="inlineStr">
@@ -23132,7 +23266,12 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>CEP DISCHARGE VALVE</t>
+          <t>MOV MAIN STEAM DRAIN STG-2</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D744" t="inlineStr">
@@ -23141,7 +23280,7 @@
         </is>
       </c>
       <c r="E744" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H744" t="n">
         <v>0</v>
@@ -23155,7 +23294,7 @@
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>MOV MAIN STEAM DRAIN STG-2</t>
+          <t>ACTUATOR ON/OFF NRV STEAM EXTRACTION 1, 2, 3</t>
         </is>
       </c>
       <c r="D745" t="inlineStr">
@@ -23173,12 +23312,12 @@
     <row r="746">
       <c r="A746" t="inlineStr">
         <is>
-          <t>WO-100826-0045</t>
+          <t>WO-100826-0063</t>
         </is>
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>ACTUATOR ON/OFF NRV STEAM EXTRACTION 1, 2, 3</t>
+          <t>ACTUATOR ON/OFF VALVE CEP-1 &amp; CEP-2</t>
         </is>
       </c>
       <c r="D746" t="inlineStr">
@@ -23196,12 +23335,17 @@
     <row r="747">
       <c r="A747" t="inlineStr">
         <is>
-          <t>WO-100826-0063</t>
+          <t>WO-100826-0037</t>
         </is>
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>ACTUATOR ON/OFF VALVE CEP-1 &amp; CEP-2</t>
+          <t>ACTUATOR MOV INLET ECONOMIZER</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D747" t="inlineStr">
@@ -23210,7 +23354,7 @@
         </is>
       </c>
       <c r="E747" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H747" t="n">
         <v>0</v>
@@ -23224,7 +23368,12 @@
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>ACTUATOR MOV INLET ECONOMIZER</t>
+          <t>ACTUATOR MOV RECIRCULATION ECONOMIZER</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D748" t="inlineStr">
@@ -23242,21 +23391,21 @@
     <row r="749">
       <c r="A749" t="inlineStr">
         <is>
-          <t>WO-100826-0037</t>
+          <t>WO-100826-0045</t>
         </is>
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>ACTUATOR MOV RECIRCULATION ECONOMIZER</t>
+          <t>10MAA10CP001: PRESSURE BEHIND TURBINE CONTROL</t>
         </is>
       </c>
       <c r="D749" t="inlineStr">
         <is>
-          <t>MSW</t>
+          <t>JAPA</t>
         </is>
       </c>
       <c r="E749" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H749" t="n">
         <v>0</v>
@@ -23270,7 +23419,7 @@
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>10MAA10CP001: PRESSURE BEHIND TURBINE CONTROL</t>
+          <t>10MAX45CP004: VALVE BLOCK, OUTLET POSITION LIVE STEAM</t>
         </is>
       </c>
       <c r="D750" t="inlineStr">
@@ -23288,12 +23437,17 @@
     <row r="751">
       <c r="A751" t="inlineStr">
         <is>
-          <t>WO-100826-0045</t>
+          <t>WO-100826-0039</t>
         </is>
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>10MAX45CP004: VALVE BLOCK, OUTLET POSITION LIVE STEAM</t>
+          <t>10HAH46CT001: TEMPERATURE AFTER DESH 2</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="D751" t="inlineStr">
@@ -23302,7 +23456,7 @@
         </is>
       </c>
       <c r="E751" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H751" t="n">
         <v>0</v>
@@ -23316,7 +23470,12 @@
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>10HAH46CT001: TEMPERATURE AFTER DESH 2</t>
+          <t>10HAH36CT0010: TEMPERATURE BEFORE DESH 2</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>30/08/2026</t>
         </is>
       </c>
       <c r="D752" t="inlineStr">
@@ -23334,12 +23493,17 @@
     <row r="753">
       <c r="A753" t="inlineStr">
         <is>
-          <t>WO-100826-0039</t>
+          <t>WO-100826-0038</t>
         </is>
       </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>10HAH36CT0010: TEMPERATURE BEFORE DESH 2</t>
+          <t>10HAH46CT010: TEMPERATURE AFTER DESH 1</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="D753" t="inlineStr">
@@ -23348,7 +23512,7 @@
         </is>
       </c>
       <c r="E753" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H753" t="n">
         <v>0</v>
@@ -23357,12 +23521,12 @@
     <row r="754">
       <c r="A754" t="inlineStr">
         <is>
-          <t>WO-100826-0038</t>
+          <t>WO-100826-0160</t>
         </is>
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>10HAH46CT010: TEMPERATURE AFTER DESH 1</t>
+          <t>10HNA11CT001: CYCLONE OUTLET TEMPERATURE</t>
         </is>
       </c>
       <c r="D754" t="inlineStr">
@@ -23380,12 +23544,12 @@
     <row r="755">
       <c r="A755" t="inlineStr">
         <is>
-          <t>WO-100826-0160</t>
+          <t>WO-100826-0030</t>
         </is>
       </c>
       <c r="B755" t="inlineStr">
         <is>
-          <t>10HNA11CT001: CYCLONE OUTLET TEMPERATURE</t>
+          <t>10HJF13CP302: LDO PRESSURE LOW TRIP FOR LANCES</t>
         </is>
       </c>
       <c r="D755" t="inlineStr">
@@ -23408,7 +23572,7 @@
       </c>
       <c r="B756" t="inlineStr">
         <is>
-          <t>10HJF13CP302: LDO PRESSURE LOW TRIP FOR LANCES</t>
+          <t>10HJF13CP303: LDO PRESSURE HIGH TRIP FOR LANCES</t>
         </is>
       </c>
       <c r="D756" t="inlineStr">
@@ -23426,12 +23590,12 @@
     <row r="757">
       <c r="A757" t="inlineStr">
         <is>
-          <t>WO-100826-0030</t>
+          <t>WO-100826-0035</t>
         </is>
       </c>
       <c r="B757" t="inlineStr">
         <is>
-          <t>10HJF13CP303: LDO PRESSURE HIGH TRIP FOR LANCES</t>
+          <t>10HJG89CP301: LPG GAS PRESSURE BEFORE MTV</t>
         </is>
       </c>
       <c r="D757" t="inlineStr">
@@ -23454,7 +23618,7 @@
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>10HJG89CP301: LPG GAS PRESSURE BEFORE MTV</t>
+          <t>10HLB01CP101: DP SWITCH ACRROS LO TANK FOR PA FAN-1</t>
         </is>
       </c>
       <c r="D758" t="inlineStr">
@@ -23477,7 +23641,7 @@
       </c>
       <c r="B759" t="inlineStr">
         <is>
-          <t>10HLB01CP101: DP SWITCH ACRROS LO TANK FOR PA FAN-1</t>
+          <t>10HLB02CP101: DP SWITCH ACRROS LO TANK FOR SA FAN-1</t>
         </is>
       </c>
       <c r="D759" t="inlineStr">
@@ -23500,7 +23664,7 @@
       </c>
       <c r="B760" t="inlineStr">
         <is>
-          <t>10HLB02CP101: DP SWITCH ACRROS LO TANK FOR SA FAN-1</t>
+          <t>10LAC10CP101: DP SWITCH BFP 1</t>
         </is>
       </c>
       <c r="D760" t="inlineStr">
@@ -23518,12 +23682,12 @@
     <row r="761">
       <c r="A761" t="inlineStr">
         <is>
-          <t>WO-100826-0035</t>
+          <t>WO-100826-0036</t>
         </is>
       </c>
       <c r="B761" t="inlineStr">
         <is>
-          <t>10LAC10CP101: DP SWITCH BFP 1</t>
+          <t>10LAC30CP101: DP SWITCH BFP 2</t>
         </is>
       </c>
       <c r="D761" t="inlineStr">
@@ -23541,21 +23705,26 @@
     <row r="762">
       <c r="A762" t="inlineStr">
         <is>
-          <t>WO-100826-0036</t>
+          <t>WO-100826-0038</t>
         </is>
       </c>
       <c r="B762" t="inlineStr">
         <is>
-          <t>10LAC30CP101: DP SWITCH BFP 2</t>
+          <t>ACTUATOR DESH-1 SPRAY WATER CONTROL VALVE</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>29/08/2026</t>
         </is>
       </c>
       <c r="D762" t="inlineStr">
         <is>
-          <t>JAPA</t>
+          <t>AMP</t>
         </is>
       </c>
       <c r="E762" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H762" t="n">
         <v>0</v>
@@ -23564,26 +23733,21 @@
     <row r="763">
       <c r="A763" t="inlineStr">
         <is>
-          <t>WO-100826-0038</t>
+          <t>WO-100826-0045</t>
         </is>
       </c>
       <c r="B763" t="inlineStr">
         <is>
-          <t>ACTUATOR DESH-1 SPRAY WATER CONTROL VALVE</t>
-        </is>
-      </c>
-      <c r="C763" t="inlineStr">
-        <is>
-          <t>29/08/2026</t>
+          <t>MOV DISCHARGE BFP-1</t>
         </is>
       </c>
       <c r="D763" t="inlineStr">
         <is>
-          <t>AMP</t>
+          <t>MSW</t>
         </is>
       </c>
       <c r="E763" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H763" t="n">
         <v>0</v>
@@ -23592,12 +23756,12 @@
     <row r="764">
       <c r="A764" t="inlineStr">
         <is>
-          <t>WO-100826-0045</t>
+          <t>WO-100826-0067</t>
         </is>
       </c>
       <c r="B764" t="inlineStr">
         <is>
-          <t>MOV DISCHARGE BFP-1</t>
+          <t>SOOT BLOWER CONTROL VALVE</t>
         </is>
       </c>
       <c r="D764" t="inlineStr">
@@ -23615,12 +23779,12 @@
     <row r="765">
       <c r="A765" t="inlineStr">
         <is>
-          <t>WO-100826-0067</t>
+          <t>WO-100826-0045</t>
         </is>
       </c>
       <c r="B765" t="inlineStr">
         <is>
-          <t>SOOT BLOWER CONTROL VALVE</t>
+          <t>ACTUATOR MOV TURBINE STOP VALVE</t>
         </is>
       </c>
       <c r="D765" t="inlineStr">
@@ -23638,21 +23802,26 @@
     <row r="766">
       <c r="A766" t="inlineStr">
         <is>
-          <t>WO-100826-0045</t>
+          <t>WO-100826-0035</t>
         </is>
       </c>
       <c r="B766" t="inlineStr">
         <is>
-          <t>ACTUATOR MOV TURBINE STOP VALVE</t>
+          <t>10QEB10CP001: P&amp;S BLOWER PRESS OUTLET</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="D766" t="inlineStr">
         <is>
-          <t>MSW</t>
+          <t>JAPA</t>
         </is>
       </c>
       <c r="E766" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H766" t="n">
         <v>0</v>
@@ -23661,12 +23830,12 @@
     <row r="767">
       <c r="A767" t="inlineStr">
         <is>
-          <t>WO-100826-0035</t>
+          <t>WO-100826-0038</t>
         </is>
       </c>
       <c r="B767" t="inlineStr">
         <is>
-          <t>10QEB10CP001: P&amp;S BLOWER PRESS OUTLET</t>
+          <t>10LAE10CF001: DESH 1 SPRAY WATER FLOW</t>
         </is>
       </c>
       <c r="C767" t="inlineStr">
@@ -23689,12 +23858,12 @@
     <row r="768">
       <c r="A768" t="inlineStr">
         <is>
-          <t>WO-100826-0038</t>
+          <t>WO-100826-0045</t>
         </is>
       </c>
       <c r="B768" t="inlineStr">
         <is>
-          <t>10LAE10CF001: DESH 1 SPRAY WATER FLOW</t>
+          <t>10LAA10CP001: FEEDWATER STORAGE TANK PRESSURE</t>
         </is>
       </c>
       <c r="D768" t="inlineStr">
@@ -23717,7 +23886,7 @@
       </c>
       <c r="B769" t="inlineStr">
         <is>
-          <t>10LAA10CP001: FEEDWATER STORAGE TANK PRESSURE</t>
+          <t>10HGC10CF001: CYCLE MAKE UP PUMP DEAERATOR</t>
         </is>
       </c>
       <c r="D769" t="inlineStr">
@@ -23740,7 +23909,7 @@
       </c>
       <c r="B770" t="inlineStr">
         <is>
-          <t>10HGC10CF001: CYCLE MAKE UP PUMP DEAERATOR</t>
+          <t>10LAA10CL001: DEAERATOR TANK LEVEL 1</t>
         </is>
       </c>
       <c r="D770" t="inlineStr">
@@ -23763,7 +23932,7 @@
       </c>
       <c r="B771" t="inlineStr">
         <is>
-          <t>10LAA10CL001: DEAERATOR TANK LEVEL 1</t>
+          <t>10LBD10CP001: TURBINE EXTRACTION III TO DEAERATOR PRESSURE</t>
         </is>
       </c>
       <c r="D771" t="inlineStr">
@@ -23786,7 +23955,7 @@
       </c>
       <c r="B772" t="inlineStr">
         <is>
-          <t>10LBD10CP001: TURBINE EXTRACTION III TO DEAERATOR PRESSURE</t>
+          <t>10MAA10CP002: TURBINE EXHAUST PRESSURE</t>
         </is>
       </c>
       <c r="D772" t="inlineStr">
@@ -23809,7 +23978,7 @@
       </c>
       <c r="B773" t="inlineStr">
         <is>
-          <t>10MAA10CP002: TURBINE EXHAUST PRESSURE</t>
+          <t>10LAA10CT001: FEEDWATER STORAGE TANK</t>
         </is>
       </c>
       <c r="D773" t="inlineStr">
@@ -23832,7 +24001,7 @@
       </c>
       <c r="B774" t="inlineStr">
         <is>
-          <t>10LAA10CT001: FEEDWATER STORAGE TANK</t>
+          <t>10LCC10CT001: LPH II - TUBE SIDE OUTLET TO DEAERATOR TEMP</t>
         </is>
       </c>
       <c r="D774" t="inlineStr">
@@ -23855,7 +24024,7 @@
       </c>
       <c r="B775" t="inlineStr">
         <is>
-          <t>10LCC10CT001: LPH II - TUBE SIDE OUTLET TO DEAERATOR TEMP</t>
+          <t>10LBS10CT001: TURBINE EXTRACTION I TO LPH1 TEMP</t>
         </is>
       </c>
       <c r="D775" t="inlineStr">
@@ -23873,12 +24042,12 @@
     <row r="776">
       <c r="A776" t="inlineStr">
         <is>
-          <t>WO-100826-0045</t>
+          <t>WO-100826-0030</t>
         </is>
       </c>
       <c r="B776" t="inlineStr">
         <is>
-          <t>10LBS10CT001: TURBINE EXTRACTION I TO LPH1 TEMP</t>
+          <t>10HJN13CP302: ATOM AIR PRESSURE LOW TRIP FOR LANCES</t>
         </is>
       </c>
       <c r="D776" t="inlineStr">
@@ -23896,12 +24065,17 @@
     <row r="777">
       <c r="A777" t="inlineStr">
         <is>
-          <t>WO-100826-0030</t>
+          <t>WO-100826-0035</t>
         </is>
       </c>
       <c r="B777" t="inlineStr">
         <is>
-          <t>10HJN13CP302: ATOM AIR PRESSURE LOW TRIP FOR LANCES</t>
+          <t>10LBA10CP502: ERV PRESSURE SWITCH</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="D777" t="inlineStr">
@@ -23910,7 +24084,7 @@
         </is>
       </c>
       <c r="E777" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H777" t="n">
         <v>0</v>
@@ -23919,17 +24093,17 @@
     <row r="778">
       <c r="A778" t="inlineStr">
         <is>
-          <t>WO-100826-0035</t>
+          <t>WO-100826-0074</t>
         </is>
       </c>
       <c r="B778" t="inlineStr">
         <is>
-          <t>10LBA10CP502: ERV PRESSURE SWITCH</t>
+          <t>10HBK01CP050: BACKPASS PRESSURE AFTER ECO</t>
         </is>
       </c>
       <c r="C778" t="inlineStr">
         <is>
-          <t>22/08/2026</t>
+          <t>31/08/2026</t>
         </is>
       </c>
       <c r="D778" t="inlineStr">
@@ -24087,10 +24261,10 @@
         <v>50</v>
       </c>
       <c r="J2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -24132,22 +24306,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>FINISH</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>100</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>29/08/2026</t>
-        </is>
+        <v>50</v>
       </c>
       <c r="J3" t="b">
         <v>1</v>
       </c>
       <c r="K3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -24575,17 +24744,22 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O12" t="n">
         <v>0</v>
@@ -24622,14 +24796,14 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K13" t="b">
         <v>0</v>
@@ -24669,17 +24843,22 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O14" t="n">
         <v>0</v>
@@ -24716,14 +24895,14 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K15" t="b">
         <v>0</v>
@@ -25030,17 +25209,22 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K22" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" t="n">
         <v>0</v>
@@ -25072,17 +25256,22 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O23" t="n">
         <v>0</v>
@@ -25114,17 +25303,22 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K24" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O24" t="n">
         <v>0</v>
@@ -26106,17 +26300,22 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O45" t="n">
         <v>0</v>
@@ -26148,17 +26347,22 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O46" t="n">
         <v>0</v>
@@ -26190,17 +26394,22 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O47" t="n">
         <v>0</v>
@@ -26232,17 +26441,22 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O48" t="n">
         <v>0</v>
@@ -26274,17 +26488,22 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O49" t="n">
         <v>0</v>
@@ -26316,17 +26535,22 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K50" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O50" t="n">
         <v>0</v>
@@ -26358,17 +26582,22 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K51" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O51" t="n">
         <v>0</v>
@@ -26912,17 +27141,22 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>FINISH</t>
         </is>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>100</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K63" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O63" t="n">
         <v>0</v>
@@ -26959,14 +27193,14 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K64" t="b">
         <v>0</v>
@@ -27006,14 +27240,14 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K65" t="b">
         <v>0</v>
@@ -27053,14 +27287,14 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>SCHED-OK</t>
+          <t>IN PROGRESS</t>
         </is>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="J66" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K66" t="b">
         <v>0</v>
@@ -28206,6 +28440,11 @@
       <c r="H92" t="n">
         <v>100</v>
       </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="J92" t="b">
         <v>1</v>
       </c>
@@ -28247,6 +28486,11 @@
       </c>
       <c r="H93" t="n">
         <v>100</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
       </c>
       <c r="J93" t="b">
         <v>1</v>
@@ -28412,14 +28656,19 @@
           <t>-70 - 70 mbar</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
       </c>
       <c r="M3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -29268,11 +29517,19 @@
           <t>0-5000 mmH20</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
+      </c>
+      <c r="M25" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
@@ -29302,11 +29559,19 @@
           <t>0-5000 mmH20</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H26" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
+      </c>
+      <c r="M26" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
@@ -29336,11 +29601,19 @@
           <t>0-180 bar</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H27" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
+      </c>
+      <c r="M27" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
@@ -29555,11 +29828,19 @@
           <t>-70 - 70 mbar</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H33" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
         <v>0</v>
+      </c>
+      <c r="M33" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -29589,11 +29870,19 @@
           <t>0.00 - 160.00 bar</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
+      </c>
+      <c r="M34" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
@@ -29701,11 +29990,19 @@
           <t>-70 - 70 mbar</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H37" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
+      </c>
+      <c r="M37" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -29735,11 +30032,19 @@
           <t>-910 - 0 mmH20</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H38" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
         <v>0</v>
+      </c>
+      <c r="M38" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="39">
@@ -29769,11 +30074,19 @@
           <t>-910 - 0 mmH20</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" t="n">
         <v>0</v>
+      </c>
+      <c r="M39" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
@@ -29803,11 +30116,19 @@
           <t>-910 - 0 mmH20</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L40" t="n">
         <v>0</v>
+      </c>
+      <c r="M40" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="41">
@@ -29949,11 +30270,19 @@
           <t>0 - 160 Bar</t>
         </is>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
         <v>0</v>
+      </c>
+      <c r="M44" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
@@ -29983,11 +30312,19 @@
           <t>0 - 160 Bar</t>
         </is>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" t="n">
         <v>0</v>
+      </c>
+      <c r="M45" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -30017,11 +30354,19 @@
           <t>0 - 160 Bar</t>
         </is>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
+      </c>
+      <c r="M46" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
@@ -30155,7 +30500,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>29/8/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="H50" t="b">
@@ -30163,6 +30508,9 @@
       </c>
       <c r="L50" t="n">
         <v>0</v>
+      </c>
+      <c r="M50" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
@@ -30194,7 +30542,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>29/8/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="H51" t="b">
@@ -30202,6 +30550,9 @@
       </c>
       <c r="L51" t="n">
         <v>0</v>
+      </c>
+      <c r="M51" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
@@ -30233,7 +30584,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>29/8/2026</t>
+          <t>22/08/2026</t>
         </is>
       </c>
       <c r="H52" t="b">
@@ -30241,6 +30592,9 @@
       </c>
       <c r="L52" t="n">
         <v>0</v>
+      </c>
+      <c r="M52" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="53">
@@ -30780,11 +31134,19 @@
           <t>0 -25 Bar</t>
         </is>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H68" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L68" t="n">
         <v>0</v>
+      </c>
+      <c r="M68" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -30814,11 +31176,19 @@
           <t>0 -25 Bar</t>
         </is>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H69" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L69" t="n">
         <v>0</v>
+      </c>
+      <c r="M69" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="70">
@@ -30848,11 +31218,19 @@
           <t>0 -25 Bar</t>
         </is>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>31/08/2026</t>
+        </is>
+      </c>
       <c r="H70" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L70" t="n">
         <v>0</v>
+      </c>
+      <c r="M70" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="71">
@@ -33490,17 +33868,7 @@
         </is>
       </c>
       <c r="N16" t="b">
-        <v>1</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="T16" t="n">
         <v>0</v>
@@ -33544,17 +33912,7 @@
         </is>
       </c>
       <c r="N17" t="b">
-        <v>1</v>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
-      <c r="P17" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="T17" t="n">
         <v>0</v>
@@ -33686,17 +34044,7 @@
         </is>
       </c>
       <c r="N20" t="b">
-        <v>1</v>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
-      <c r="P20" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="T20" t="n">
         <v>0</v>
@@ -33740,17 +34088,7 @@
         </is>
       </c>
       <c r="N21" t="b">
-        <v>1</v>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="T21" t="n">
         <v>0</v>
@@ -33882,17 +34220,7 @@
         </is>
       </c>
       <c r="N24" t="b">
-        <v>1</v>
-      </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
-      <c r="P24" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="T24" t="n">
         <v>0</v>
@@ -33936,17 +34264,7 @@
         </is>
       </c>
       <c r="N25" t="b">
-        <v>1</v>
-      </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="T25" t="n">
         <v>0</v>
@@ -34078,17 +34396,7 @@
         </is>
       </c>
       <c r="N28" t="b">
-        <v>1</v>
-      </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
-      <c r="P28" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="T28" t="n">
         <v>0</v>
@@ -34132,17 +34440,7 @@
         </is>
       </c>
       <c r="N29" t="b">
-        <v>1</v>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
-        <is>
-          <t>22/08/2026</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="T29" t="n">
         <v>0</v>

</xml_diff>